<commit_message>
📊 Hybrid MF Ranker Week-27 - 30-Jun-2026 09:30 PM IST
</commit_message>
<xml_diff>
--- a/output/mf_ranked_hybrid.xlsx
+++ b/output/mf_ranked_hybrid.xlsx
@@ -1703,7 +1703,7 @@
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2">
-        <f>"All Funds Consolidated | 55% Momentum + 45% Quality | ✅ Full: "&amp;COUNTIF($U:$U,"FULL")&amp;" | ⚠️ Momentum: "&amp;COUNTIF($U:$U,"MOMENTUM_ONLY")&amp;" | ❌ Missing: "&amp;COUNTIF($U:$U,"MISSING")&amp;" | Total: "&amp;(COUNTA($B:$B)-4)</f>
+        <f>"All Funds Consolidated | 55% Momentum + 45% Quality | ✅ Full: "&amp;COUNTIF($U:$U,"FULL")&amp;" | ⚠️ Momentum: "&amp;COUNTIF($U:$U,"MOMENTUM_ONLY")&amp;" | ❌ Missing: "&amp;COUNTIF($U:$U,"MISSING")&amp;" | Total: "&amp;COUNTA(B5:B211)</f>
         <v/>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="B22" s="79" t="inlineStr">
         <is>
-          <t>Nippon India Balanced Advantage Fund-Growth Plan-Growth Option</t>
+          <t>Nippon India Balanced Advantage Fund-Growth Plan-Bonus Option</t>
         </is>
       </c>
       <c r="C22" s="79" t="inlineStr">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="B23" s="83" t="inlineStr">
         <is>
-          <t>Nippon India Balanced Advantage Fund-Growth Plan-Bonus Option</t>
+          <t>Nippon India Balanced Advantage Fund-Growth Plan-Growth Option</t>
         </is>
       </c>
       <c r="C23" s="83" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="B71" s="83" t="inlineStr">
         <is>
-          <t>TATA Arbitrage Fund Regular Plan - Monthly Reinvestment of Income Distribution cum capital withdrawal option</t>
+          <t>TATA Arbitrage Fund Regular Plan - Monthly Payout of Income Distribution cum capital withdrawal option</t>
         </is>
       </c>
       <c r="C71" s="83" t="inlineStr">
@@ -7507,7 +7507,7 @@
       </c>
       <c r="B72" s="79" t="inlineStr">
         <is>
-          <t>Tata Arbitrage Fund-Regular Plan-Growth</t>
+          <t>TATA Arbitrage Fund Regular Plan - Monthly Reinvestment of Income Distribution cum capital withdrawal option</t>
         </is>
       </c>
       <c r="C72" s="79" t="inlineStr">
@@ -7541,7 +7541,7 @@
         <v>6.400187969758764</v>
       </c>
       <c r="K72" s="80" t="n">
-        <v>21.85</v>
+        <v>21.86</v>
       </c>
       <c r="L72" s="88" t="n">
         <v>58.9</v>
@@ -7591,7 +7591,7 @@
       </c>
       <c r="B73" s="83" t="inlineStr">
         <is>
-          <t>TATA Arbitrage Fund Regular Plan - Monthly Payout of Income Distribution cum capital withdrawal option</t>
+          <t>Tata Arbitrage Fund-Regular Plan-Growth</t>
         </is>
       </c>
       <c r="C73" s="83" t="inlineStr">
@@ -7625,7 +7625,7 @@
         <v>6.400187969758764</v>
       </c>
       <c r="K73" s="84" t="n">
-        <v>21.86</v>
+        <v>21.85</v>
       </c>
       <c r="L73" s="88" t="n">
         <v>58.9</v>
@@ -7927,12 +7927,12 @@
       </c>
       <c r="B77" s="83" t="inlineStr">
         <is>
-          <t>Union Balanced Advantage Fund - Regular Plan - Growth Option</t>
+          <t>Axis Balanced Advantage Fund - Regular Plan - Growth</t>
         </is>
       </c>
       <c r="C77" s="83" t="inlineStr">
         <is>
-          <t>Union Mutual Fund</t>
+          <t>Axis Mutual Fund</t>
         </is>
       </c>
       <c r="D77" s="83" t="inlineStr">
@@ -7946,22 +7946,22 @@
         </is>
       </c>
       <c r="F77" s="84" t="n">
-        <v>1.8</v>
+        <v>1.67</v>
       </c>
       <c r="G77" s="84" t="n">
-        <v>5.83</v>
+        <v>5.37</v>
       </c>
       <c r="H77" s="86" t="n">
-        <v>-1.07</v>
+        <v>-0.88</v>
       </c>
       <c r="I77" s="84" t="n">
-        <v>0.1</v>
+        <v>1.09</v>
       </c>
       <c r="J77" s="84" t="n">
-        <v>2.4987804805501</v>
+        <v>4.713895925994471</v>
       </c>
       <c r="K77" s="84" t="n">
-        <v>26.65</v>
+        <v>40.96</v>
       </c>
       <c r="L77" s="88" t="n">
         <v>57.8</v>
@@ -8011,12 +8011,12 @@
       </c>
       <c r="B78" s="79" t="inlineStr">
         <is>
-          <t>Axis Balanced Advantage Fund - Regular Plan - Growth</t>
+          <t>Union Balanced Advantage Fund - Regular Plan - Growth Option</t>
         </is>
       </c>
       <c r="C78" s="79" t="inlineStr">
         <is>
-          <t>Axis Mutual Fund</t>
+          <t>Union Mutual Fund</t>
         </is>
       </c>
       <c r="D78" s="79" t="inlineStr">
@@ -8030,22 +8030,22 @@
         </is>
       </c>
       <c r="F78" s="80" t="n">
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="G78" s="80" t="n">
-        <v>5.37</v>
+        <v>5.83</v>
       </c>
       <c r="H78" s="87" t="n">
-        <v>-0.88</v>
+        <v>-1.07</v>
       </c>
       <c r="I78" s="80" t="n">
-        <v>1.09</v>
+        <v>0.1</v>
       </c>
       <c r="J78" s="80" t="n">
-        <v>4.713895925994471</v>
+        <v>2.4987804805501</v>
       </c>
       <c r="K78" s="80" t="n">
-        <v>40.96</v>
+        <v>26.65</v>
       </c>
       <c r="L78" s="88" t="n">
         <v>57.8</v>
@@ -12379,7 +12379,7 @@
       </c>
       <c r="B130" s="79" t="inlineStr">
         <is>
-          <t>Nippon India Equity Savings Fund- Growth Plan- Growth Option</t>
+          <t>Nippon India Equity Savings Fund- Growth Plan- Bonus Option</t>
         </is>
       </c>
       <c r="C130" s="79" t="inlineStr">
@@ -12463,7 +12463,7 @@
       </c>
       <c r="B131" s="83" t="inlineStr">
         <is>
-          <t>Nippon India Equity Savings Fund- Growth Plan- Bonus Option</t>
+          <t>Nippon India Equity Savings Fund- Growth Plan- Growth Option</t>
         </is>
       </c>
       <c r="C131" s="83" t="inlineStr">
@@ -12799,12 +12799,12 @@
       </c>
       <c r="B135" s="83" t="inlineStr">
         <is>
-          <t>ITI Balanced Advantage Fund - Regular Plan - Growth Option</t>
+          <t>PGIM India Balanced Advantage Fund - Regular Plan - Growth Option</t>
         </is>
       </c>
       <c r="C135" s="83" t="inlineStr">
         <is>
-          <t>ITI Mutual Fund</t>
+          <t>PGIM India Mutual Fund</t>
         </is>
       </c>
       <c r="D135" s="83" t="inlineStr">
@@ -12818,22 +12818,22 @@
         </is>
       </c>
       <c r="F135" s="84" t="n">
-        <v>1.11</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="G135" s="84" t="n">
-        <v>4.28</v>
+        <v>5.64</v>
       </c>
       <c r="H135" s="86" t="n">
-        <v>-3.66</v>
+        <v>-3.29</v>
       </c>
       <c r="I135" s="86" t="n">
-        <v>-2.89</v>
+        <v>-3.97</v>
       </c>
       <c r="J135" s="84" t="n">
-        <v>1.602165331256589</v>
+        <v>1.533245786786508</v>
       </c>
       <c r="K135" s="84" t="n">
-        <v>27.39</v>
+        <v>21.18</v>
       </c>
       <c r="L135" s="89" t="n">
         <v>25.1</v>
@@ -12883,12 +12883,12 @@
       </c>
       <c r="B136" s="79" t="inlineStr">
         <is>
-          <t>PGIM India Balanced Advantage Fund - Regular Plan - Growth Option</t>
+          <t>ITI Balanced Advantage Fund - Regular Plan - Growth Option</t>
         </is>
       </c>
       <c r="C136" s="79" t="inlineStr">
         <is>
-          <t>PGIM India Mutual Fund</t>
+          <t>ITI Mutual Fund</t>
         </is>
       </c>
       <c r="D136" s="79" t="inlineStr">
@@ -12902,22 +12902,22 @@
         </is>
       </c>
       <c r="F136" s="80" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.11</v>
       </c>
       <c r="G136" s="80" t="n">
-        <v>5.64</v>
+        <v>4.28</v>
       </c>
       <c r="H136" s="87" t="n">
-        <v>-3.29</v>
+        <v>-3.66</v>
       </c>
       <c r="I136" s="87" t="n">
-        <v>-3.97</v>
+        <v>-2.89</v>
       </c>
       <c r="J136" s="80" t="n">
-        <v>1.533245786786508</v>
+        <v>1.602165331256589</v>
       </c>
       <c r="K136" s="80" t="n">
-        <v>21.18</v>
+        <v>27.39</v>
       </c>
       <c r="L136" s="89" t="n">
         <v>25.1</v>
@@ -13723,7 +13723,7 @@
       </c>
       <c r="B146" s="79" t="inlineStr">
         <is>
-          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- Monthly - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment.</t>
+          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- Quarterly - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment)</t>
         </is>
       </c>
       <c r="C146" s="79" t="inlineStr">
@@ -13807,7 +13807,7 @@
       </c>
       <c r="B147" s="83" t="inlineStr">
         <is>
-          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment)</t>
+          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund) - Regular Plan - Growth option</t>
         </is>
       </c>
       <c r="C147" s="83" t="inlineStr">
@@ -13841,7 +13841,7 @@
         <v>-0.6873623348971791</v>
       </c>
       <c r="K147" s="84" t="n">
-        <v>29.08</v>
+        <v>29.07</v>
       </c>
       <c r="L147" s="89" t="n">
         <v>14.9</v>
@@ -13891,7 +13891,7 @@
       </c>
       <c r="B148" s="79" t="inlineStr">
         <is>
-          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund) - Regular Plan - Growth option</t>
+          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- Half Yearly - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment)</t>
         </is>
       </c>
       <c r="C148" s="79" t="inlineStr">
@@ -13925,7 +13925,7 @@
         <v>-0.6873623348971791</v>
       </c>
       <c r="K148" s="80" t="n">
-        <v>29.07</v>
+        <v>29.08</v>
       </c>
       <c r="L148" s="89" t="n">
         <v>14.9</v>
@@ -13975,7 +13975,7 @@
       </c>
       <c r="B149" s="83" t="inlineStr">
         <is>
-          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- Half Yearly - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment)</t>
+          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- Monthly - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment.</t>
         </is>
       </c>
       <c r="C149" s="83" t="inlineStr">
@@ -14059,7 +14059,7 @@
       </c>
       <c r="B150" s="79" t="inlineStr">
         <is>
-          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- Quarterly - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment)</t>
+          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment)</t>
         </is>
       </c>
       <c r="C150" s="79" t="inlineStr">
@@ -14143,7 +14143,7 @@
       </c>
       <c r="B151" s="83" t="inlineStr">
         <is>
-          <t>TATA Balanced Advantage Fund Regular Plan - Reinvestment of Income Distribution cum capital withdrawal option</t>
+          <t>TATA Balanced Advantage Fund Regular Plan - Payout of Income Distribution cum capital withdrawal option</t>
         </is>
       </c>
       <c r="C151" s="83" t="inlineStr">
@@ -14227,7 +14227,7 @@
       </c>
       <c r="B152" s="79" t="inlineStr">
         <is>
-          <t>TATA Balanced Advantage Fund Regular Plan - Payout of Income Distribution cum capital withdrawal option</t>
+          <t>TATA Balanced Advantage Fund Regular Plan - Reinvestment of Income Distribution cum capital withdrawal option</t>
         </is>
       </c>
       <c r="C152" s="79" t="inlineStr">
@@ -14731,38 +14731,38 @@
       </c>
       <c r="B158" s="26" t="inlineStr">
         <is>
-          <t>quant Arbitrage Fund - Growth Option - Regular Plan</t>
+          <t>360 ONE Balanced Hybrid Fund - Regular Plan - Growth</t>
         </is>
       </c>
       <c r="C158" s="26" t="inlineStr">
         <is>
-          <t>quant Mutual Fund</t>
+          <t>360 ONE Mutual Fund</t>
         </is>
       </c>
       <c r="D158" s="26" t="inlineStr">
         <is>
-          <t>Arbitrage Fund</t>
+          <t>Balanced Hybrid Fund</t>
         </is>
       </c>
       <c r="E158" s="26" t="inlineStr">
         <is>
-          <t>Arbitrage Fund</t>
+          <t>Balanced Hybrid Fund</t>
         </is>
       </c>
       <c r="F158" s="27" t="n">
-        <v>0.85</v>
+        <v>2.57</v>
       </c>
       <c r="G158" s="27" t="n">
-        <v>1.63</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="H158" s="27" t="n">
-        <v>3.47</v>
+        <v>2.71</v>
       </c>
       <c r="I158" s="27" t="n">
-        <v>6.84</v>
+        <v>2.84</v>
       </c>
       <c r="J158" s="27" t="n">
-        <v>0</v>
+        <v>4.244903952183687</v>
       </c>
       <c r="K158" s="27" t="n">
         <v>0</v>
@@ -14815,38 +14815,38 @@
       </c>
       <c r="B159" s="26" t="inlineStr">
         <is>
-          <t>360 ONE Balanced Hybrid Fund - Regular Plan - Growth</t>
+          <t>quant Arbitrage Fund - Growth Option - Regular Plan</t>
         </is>
       </c>
       <c r="C159" s="26" t="inlineStr">
         <is>
-          <t>360 ONE Mutual Fund</t>
+          <t>quant Mutual Fund</t>
         </is>
       </c>
       <c r="D159" s="26" t="inlineStr">
         <is>
-          <t>Balanced Hybrid Fund</t>
+          <t>Arbitrage Fund</t>
         </is>
       </c>
       <c r="E159" s="26" t="inlineStr">
         <is>
-          <t>Balanced Hybrid Fund</t>
+          <t>Arbitrage Fund</t>
         </is>
       </c>
       <c r="F159" s="27" t="n">
-        <v>2.57</v>
+        <v>0.85</v>
       </c>
       <c r="G159" s="27" t="n">
-        <v>8.220000000000001</v>
+        <v>1.63</v>
       </c>
       <c r="H159" s="27" t="n">
-        <v>2.71</v>
+        <v>3.47</v>
       </c>
       <c r="I159" s="27" t="n">
-        <v>2.84</v>
+        <v>6.84</v>
       </c>
       <c r="J159" s="27" t="n">
-        <v>4.244903952183687</v>
+        <v>0</v>
       </c>
       <c r="K159" s="27" t="n">
         <v>0</v>
@@ -18427,29 +18427,29 @@
       </c>
       <c r="B202" s="91" t="inlineStr">
         <is>
-          <t>Helios Arbitrage Fund - Regular Growth</t>
+          <t>Nippon India Equity Savings Fund - Segregated Portfolio 2 - Growth Plan - Bonus Option</t>
         </is>
       </c>
       <c r="C202" s="91" t="inlineStr">
         <is>
-          <t>Helios Mutual Fund</t>
+          <t>Nippon India Mutual Fund</t>
         </is>
       </c>
       <c r="D202" s="91" t="inlineStr">
         <is>
-          <t>Arbitrage Fund</t>
+          <t>Equity Savings</t>
         </is>
       </c>
       <c r="E202" s="91" t="inlineStr">
         <is>
-          <t>Arbitrage Fund</t>
+          <t>Equity Savings</t>
         </is>
       </c>
       <c r="F202" s="92" t="n">
-        <v>0.6899999999999999</v>
+        <v>0</v>
       </c>
       <c r="G202" s="92" t="n">
-        <v>1.4</v>
+        <v>0</v>
       </c>
       <c r="H202" s="92" t="n">
         <v>0</v>
@@ -18511,12 +18511,12 @@
       </c>
       <c r="B203" s="91" t="inlineStr">
         <is>
-          <t>Kotak Multi Asset Active FOF - Regular - Growth</t>
+          <t>Capitalmind Multi Asset Allocation Fund-Regular-Growth</t>
         </is>
       </c>
       <c r="C203" s="91" t="inlineStr">
         <is>
-          <t>Kotak Mahindra Mutual Fund</t>
+          <t>Capitalmind Mutual Fund</t>
         </is>
       </c>
       <c r="D203" s="91" t="inlineStr">
@@ -18530,10 +18530,10 @@
         </is>
       </c>
       <c r="F203" s="102" t="n">
-        <v>-1.52</v>
-      </c>
-      <c r="G203" s="92" t="n">
-        <v>0</v>
+        <v>-5.32</v>
+      </c>
+      <c r="G203" s="102" t="n">
+        <v>-2.33</v>
       </c>
       <c r="H203" s="92" t="n">
         <v>0</v>
@@ -18595,26 +18595,26 @@
       </c>
       <c r="B204" s="91" t="inlineStr">
         <is>
-          <t>Groww Arbitrage Fund Regular Growth</t>
+          <t>Kotak Multi Asset Active FOF - Regular - Growth</t>
         </is>
       </c>
       <c r="C204" s="91" t="inlineStr">
         <is>
-          <t>Groww Mutual Fund</t>
+          <t>Kotak Mahindra Mutual Fund</t>
         </is>
       </c>
       <c r="D204" s="91" t="inlineStr">
         <is>
-          <t>Arbitrage Fund</t>
+          <t>Multi Asset Allocation</t>
         </is>
       </c>
       <c r="E204" s="91" t="inlineStr">
         <is>
-          <t>Arbitrage Fund</t>
-        </is>
-      </c>
-      <c r="F204" s="92" t="n">
-        <v>0.6</v>
+          <t>Multi Asset Allocation</t>
+        </is>
+      </c>
+      <c r="F204" s="102" t="n">
+        <v>-1.52</v>
       </c>
       <c r="G204" s="92" t="n">
         <v>0</v>
@@ -18679,7 +18679,7 @@
       </c>
       <c r="B205" s="91" t="inlineStr">
         <is>
-          <t>Nippon India Aggressive Hybrid Fund - Segregated Portfolio 2 - Growth Plan</t>
+          <t>Nippon India Conservative Hybrid  Fund - Segregated Portfolio 2 - Growth Plan</t>
         </is>
       </c>
       <c r="C205" s="91" t="inlineStr">
@@ -18689,12 +18689,12 @@
       </c>
       <c r="D205" s="91" t="inlineStr">
         <is>
-          <t>Aggressive Hybrid Fund</t>
+          <t>Conservative Hybrid Fund</t>
         </is>
       </c>
       <c r="E205" s="91" t="inlineStr">
         <is>
-          <t>Aggressive Hybrid Fund</t>
+          <t>Conservative Hybrid Fund</t>
         </is>
       </c>
       <c r="F205" s="92" t="n">
@@ -18763,26 +18763,26 @@
       </c>
       <c r="B206" s="91" t="inlineStr">
         <is>
-          <t>Nippon India Equity Savings Fund - Segregated Portfolio 2 - Growth Plan - Growth Option</t>
+          <t>Groww Arbitrage Fund Regular Growth</t>
         </is>
       </c>
       <c r="C206" s="91" t="inlineStr">
         <is>
-          <t>Nippon India Mutual Fund</t>
+          <t>Groww Mutual Fund</t>
         </is>
       </c>
       <c r="D206" s="91" t="inlineStr">
         <is>
-          <t>Equity Savings</t>
+          <t>Arbitrage Fund</t>
         </is>
       </c>
       <c r="E206" s="91" t="inlineStr">
         <is>
-          <t>Equity Savings</t>
+          <t>Arbitrage Fund</t>
         </is>
       </c>
       <c r="F206" s="92" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="G206" s="92" t="n">
         <v>0</v>
@@ -18847,29 +18847,29 @@
       </c>
       <c r="B207" s="91" t="inlineStr">
         <is>
-          <t>Nippon India Equity Savings Fund - Segregated Portfolio 2 - Growth Plan - Bonus Option</t>
+          <t>Helios Arbitrage Fund - Regular Growth</t>
         </is>
       </c>
       <c r="C207" s="91" t="inlineStr">
         <is>
-          <t>Nippon India Mutual Fund</t>
+          <t>Helios Mutual Fund</t>
         </is>
       </c>
       <c r="D207" s="91" t="inlineStr">
         <is>
-          <t>Equity Savings</t>
+          <t>Arbitrage Fund</t>
         </is>
       </c>
       <c r="E207" s="91" t="inlineStr">
         <is>
-          <t>Equity Savings</t>
+          <t>Arbitrage Fund</t>
         </is>
       </c>
       <c r="F207" s="92" t="n">
-        <v>0</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G207" s="92" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="H207" s="92" t="n">
         <v>0</v>
@@ -18931,7 +18931,7 @@
       </c>
       <c r="B208" s="91" t="inlineStr">
         <is>
-          <t>Nippon India Conservative Hybrid  Fund - Segregated Portfolio 2 - Growth Plan</t>
+          <t>Nippon India Equity Savings Fund - Segregated Portfolio 2 - Growth Plan - Growth Option</t>
         </is>
       </c>
       <c r="C208" s="91" t="inlineStr">
@@ -18941,12 +18941,12 @@
       </c>
       <c r="D208" s="91" t="inlineStr">
         <is>
-          <t>Conservative Hybrid Fund</t>
+          <t>Equity Savings</t>
         </is>
       </c>
       <c r="E208" s="91" t="inlineStr">
         <is>
-          <t>Conservative Hybrid Fund</t>
+          <t>Equity Savings</t>
         </is>
       </c>
       <c r="F208" s="92" t="n">
@@ -19015,29 +19015,29 @@
       </c>
       <c r="B209" s="91" t="inlineStr">
         <is>
-          <t>The Wealth Company Balanced Advantage Fund - Regular Growth</t>
+          <t>Capitalmind Arbitrage Fund-regular-Growth</t>
         </is>
       </c>
       <c r="C209" s="91" t="inlineStr">
         <is>
-          <t>The Wealth Company Mutual Fund</t>
+          <t>Capitalmind Mutual Fund</t>
         </is>
       </c>
       <c r="D209" s="91" t="inlineStr">
         <is>
-          <t>Dynamic Asset Allocation Or Balanced Advantage</t>
+          <t>Arbitrage Fund</t>
         </is>
       </c>
       <c r="E209" s="91" t="inlineStr">
         <is>
-          <t>Dynamic Asset Allocation Or Balanced Advantage</t>
+          <t>Arbitrage Fund</t>
         </is>
       </c>
       <c r="F209" s="92" t="n">
-        <v>0.35</v>
+        <v>0.58</v>
       </c>
       <c r="G209" s="92" t="n">
-        <v>5.17</v>
+        <v>1.26</v>
       </c>
       <c r="H209" s="92" t="n">
         <v>0</v>
@@ -19099,29 +19099,29 @@
       </c>
       <c r="B210" s="91" t="inlineStr">
         <is>
-          <t>Capitalmind Multi Asset Allocation Fund-Regular-Growth</t>
+          <t>Nippon India Aggressive Hybrid Fund - Segregated Portfolio 2 - Growth Plan</t>
         </is>
       </c>
       <c r="C210" s="91" t="inlineStr">
         <is>
-          <t>Capitalmind Mutual Fund</t>
+          <t>Nippon India Mutual Fund</t>
         </is>
       </c>
       <c r="D210" s="91" t="inlineStr">
         <is>
-          <t>Multi Asset Allocation</t>
+          <t>Aggressive Hybrid Fund</t>
         </is>
       </c>
       <c r="E210" s="91" t="inlineStr">
         <is>
-          <t>Multi Asset Allocation</t>
-        </is>
-      </c>
-      <c r="F210" s="102" t="n">
-        <v>-5.32</v>
-      </c>
-      <c r="G210" s="102" t="n">
-        <v>-2.33</v>
+          <t>Aggressive Hybrid Fund</t>
+        </is>
+      </c>
+      <c r="F210" s="92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G210" s="92" t="n">
+        <v>0</v>
       </c>
       <c r="H210" s="92" t="n">
         <v>0</v>
@@ -19183,29 +19183,29 @@
       </c>
       <c r="B211" s="91" t="inlineStr">
         <is>
-          <t>Capitalmind Arbitrage Fund-regular-Growth</t>
+          <t>The Wealth Company Balanced Advantage Fund - Regular Growth</t>
         </is>
       </c>
       <c r="C211" s="91" t="inlineStr">
         <is>
-          <t>Capitalmind Mutual Fund</t>
+          <t>The Wealth Company Mutual Fund</t>
         </is>
       </c>
       <c r="D211" s="91" t="inlineStr">
         <is>
-          <t>Arbitrage Fund</t>
+          <t>Dynamic Asset Allocation Or Balanced Advantage</t>
         </is>
       </c>
       <c r="E211" s="91" t="inlineStr">
         <is>
-          <t>Arbitrage Fund</t>
+          <t>Dynamic Asset Allocation Or Balanced Advantage</t>
         </is>
       </c>
       <c r="F211" s="92" t="n">
-        <v>0.58</v>
+        <v>0.35</v>
       </c>
       <c r="G211" s="92" t="n">
-        <v>1.26</v>
+        <v>5.17</v>
       </c>
       <c r="H211" s="92" t="n">
         <v>0</v>
@@ -19301,7 +19301,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-28 17:26:20 | Comprehensive Documentation | All Values Numeric (0 = Missing)</t>
+          <t>Generated: 2026-06-30 16:00:18 | Comprehensive Documentation | All Values Numeric (0 = Missing)</t>
         </is>
       </c>
     </row>
@@ -23585,7 +23585,7 @@
       </c>
       <c r="B34" s="79" t="inlineStr">
         <is>
-          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- Monthly - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment.</t>
+          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- Half Yearly - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment)</t>
         </is>
       </c>
       <c r="C34" s="79" t="inlineStr">
@@ -23652,7 +23652,7 @@
       </c>
       <c r="B35" s="83" t="inlineStr">
         <is>
-          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment)</t>
+          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- Quarterly - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment)</t>
         </is>
       </c>
       <c r="C35" s="83" t="inlineStr">
@@ -23719,7 +23719,7 @@
       </c>
       <c r="B36" s="79" t="inlineStr">
         <is>
-          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- Quarterly - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment)</t>
+          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- Monthly - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment.</t>
         </is>
       </c>
       <c r="C36" s="79" t="inlineStr">
@@ -23786,7 +23786,7 @@
       </c>
       <c r="B37" s="83" t="inlineStr">
         <is>
-          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund) - Regular Plan - Growth option</t>
+          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment)</t>
         </is>
       </c>
       <c r="C37" s="83" t="inlineStr">
@@ -23815,7 +23815,7 @@
         <v>-0.6873623348971791</v>
       </c>
       <c r="J37" s="84" t="n">
-        <v>29.07</v>
+        <v>29.08</v>
       </c>
       <c r="K37" s="89" t="n">
         <v>14.9</v>
@@ -23853,7 +23853,7 @@
       </c>
       <c r="B38" s="79" t="inlineStr">
         <is>
-          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund)- Regular Plan- Half Yearly - Income Distribution cum capital withdrawal Option (Payout &amp; Reinvestment)</t>
+          <t>Groww Aggressive Hybrid Fund (formerly known as Indiabulls Equity Hybrid Fund) - Regular Plan - Growth option</t>
         </is>
       </c>
       <c r="C38" s="79" t="inlineStr">
@@ -23882,7 +23882,7 @@
         <v>-0.6873623348971791</v>
       </c>
       <c r="J38" s="80" t="n">
-        <v>29.08</v>
+        <v>29.07</v>
       </c>
       <c r="K38" s="89" t="n">
         <v>14.9</v>
@@ -25383,7 +25383,7 @@
       </c>
       <c r="B22" s="79" t="inlineStr">
         <is>
-          <t>TATA Arbitrage Fund Regular Plan - Monthly Reinvestment of Income Distribution cum capital withdrawal option</t>
+          <t>TATA Arbitrage Fund Regular Plan - Monthly Payout of Income Distribution cum capital withdrawal option</t>
         </is>
       </c>
       <c r="C22" s="79" t="inlineStr">
@@ -25450,7 +25450,7 @@
       </c>
       <c r="B23" s="83" t="inlineStr">
         <is>
-          <t>TATA Arbitrage Fund Regular Plan - Monthly Payout of Income Distribution cum capital withdrawal option</t>
+          <t>Tata Arbitrage Fund-Regular Plan-Growth</t>
         </is>
       </c>
       <c r="C23" s="83" t="inlineStr">
@@ -25479,7 +25479,7 @@
         <v>6.400187969758764</v>
       </c>
       <c r="J23" s="84" t="n">
-        <v>21.86</v>
+        <v>21.85</v>
       </c>
       <c r="K23" s="88" t="n">
         <v>58.9</v>
@@ -25517,7 +25517,7 @@
       </c>
       <c r="B24" s="79" t="inlineStr">
         <is>
-          <t>Tata Arbitrage Fund-Regular Plan-Growth</t>
+          <t>TATA Arbitrage Fund Regular Plan - Monthly Reinvestment of Income Distribution cum capital withdrawal option</t>
         </is>
       </c>
       <c r="C24" s="79" t="inlineStr">
@@ -25546,7 +25546,7 @@
         <v>6.400187969758764</v>
       </c>
       <c r="J24" s="80" t="n">
-        <v>21.85</v>
+        <v>21.86</v>
       </c>
       <c r="K24" s="88" t="n">
         <v>58.9</v>
@@ -26790,12 +26790,12 @@
       </c>
       <c r="B43" s="91" t="inlineStr">
         <is>
-          <t>Helios Arbitrage Fund - Regular Growth</t>
+          <t>Capitalmind Arbitrage Fund-regular-Growth</t>
         </is>
       </c>
       <c r="C43" s="91" t="inlineStr">
         <is>
-          <t>Helios Mutual Fund</t>
+          <t>Capitalmind Mutual Fund</t>
         </is>
       </c>
       <c r="D43" s="91" t="inlineStr">
@@ -26804,10 +26804,10 @@
         </is>
       </c>
       <c r="E43" s="92" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.58</v>
       </c>
       <c r="F43" s="92" t="n">
-        <v>1.4</v>
+        <v>1.26</v>
       </c>
       <c r="G43" s="92" t="n">
         <v>0</v>
@@ -26857,12 +26857,12 @@
       </c>
       <c r="B44" s="91" t="inlineStr">
         <is>
-          <t>Groww Arbitrage Fund Regular Growth</t>
+          <t>Helios Arbitrage Fund - Regular Growth</t>
         </is>
       </c>
       <c r="C44" s="91" t="inlineStr">
         <is>
-          <t>Groww Mutual Fund</t>
+          <t>Helios Mutual Fund</t>
         </is>
       </c>
       <c r="D44" s="91" t="inlineStr">
@@ -26871,10 +26871,10 @@
         </is>
       </c>
       <c r="E44" s="92" t="n">
-        <v>0.6</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F44" s="92" t="n">
-        <v>0</v>
+        <v>1.4</v>
       </c>
       <c r="G44" s="92" t="n">
         <v>0</v>
@@ -26924,12 +26924,12 @@
       </c>
       <c r="B45" s="91" t="inlineStr">
         <is>
-          <t>Capitalmind Arbitrage Fund-regular-Growth</t>
+          <t>Groww Arbitrage Fund Regular Growth</t>
         </is>
       </c>
       <c r="C45" s="91" t="inlineStr">
         <is>
-          <t>Capitalmind Mutual Fund</t>
+          <t>Groww Mutual Fund</t>
         </is>
       </c>
       <c r="D45" s="91" t="inlineStr">
@@ -26938,10 +26938,10 @@
         </is>
       </c>
       <c r="E45" s="92" t="n">
-        <v>0.58</v>
+        <v>0.6</v>
       </c>
       <c r="F45" s="92" t="n">
-        <v>1.26</v>
+        <v>0</v>
       </c>
       <c r="G45" s="92" t="n">
         <v>0</v>
@@ -29370,7 +29370,7 @@
       </c>
       <c r="B7" s="76" t="inlineStr">
         <is>
-          <t>Nippon India Balanced Advantage Fund-Growth Plan-Bonus Option</t>
+          <t>Nippon India Balanced Advantage Fund-Growth Plan-Growth Option</t>
         </is>
       </c>
       <c r="C7" s="76" t="inlineStr">
@@ -29437,7 +29437,7 @@
       </c>
       <c r="B8" s="76" t="inlineStr">
         <is>
-          <t>Nippon India Balanced Advantage Fund-Growth Plan-Growth Option</t>
+          <t>Nippon India Balanced Advantage Fund-Growth Plan-Bonus Option</t>
         </is>
       </c>
       <c r="C8" s="76" t="inlineStr">
@@ -30107,12 +30107,12 @@
       </c>
       <c r="B18" s="79" t="inlineStr">
         <is>
-          <t>Kotak Balanced Advantage Fund -Regular Plan - Growth Option</t>
+          <t>HSBC Balanced Advantage Fund - Regular Growth</t>
         </is>
       </c>
       <c r="C18" s="79" t="inlineStr">
         <is>
-          <t>Kotak Mahindra Mutual Fund</t>
+          <t>HSBC Mutual Fund</t>
         </is>
       </c>
       <c r="D18" s="79" t="inlineStr">
@@ -30121,22 +30121,22 @@
         </is>
       </c>
       <c r="E18" s="80" t="n">
-        <v>1.47</v>
+        <v>1.96</v>
       </c>
       <c r="F18" s="80" t="n">
-        <v>6.58</v>
+        <v>5.4</v>
       </c>
       <c r="G18" s="87" t="n">
-        <v>-0.26</v>
+        <v>-0.48</v>
       </c>
       <c r="H18" s="80" t="n">
-        <v>0.79</v>
+        <v>0.89</v>
       </c>
       <c r="I18" s="80" t="n">
-        <v>4.455732250556732</v>
+        <v>3.653268158799516</v>
       </c>
       <c r="J18" s="80" t="n">
-        <v>31.65</v>
+        <v>32.05</v>
       </c>
       <c r="K18" s="88" t="n">
         <v>64.09999999999999</v>
@@ -30174,12 +30174,12 @@
       </c>
       <c r="B19" s="83" t="inlineStr">
         <is>
-          <t>HSBC Balanced Advantage Fund - Regular Growth</t>
+          <t>Kotak Balanced Advantage Fund -Regular Plan - Growth Option</t>
         </is>
       </c>
       <c r="C19" s="83" t="inlineStr">
         <is>
-          <t>HSBC Mutual Fund</t>
+          <t>Kotak Mahindra Mutual Fund</t>
         </is>
       </c>
       <c r="D19" s="83" t="inlineStr">
@@ -30188,22 +30188,22 @@
         </is>
       </c>
       <c r="E19" s="84" t="n">
-        <v>1.96</v>
+        <v>1.47</v>
       </c>
       <c r="F19" s="84" t="n">
-        <v>5.4</v>
+        <v>6.58</v>
       </c>
       <c r="G19" s="86" t="n">
-        <v>-0.48</v>
+        <v>-0.26</v>
       </c>
       <c r="H19" s="84" t="n">
-        <v>0.89</v>
+        <v>0.79</v>
       </c>
       <c r="I19" s="84" t="n">
-        <v>3.653268158799516</v>
+        <v>4.455732250556732</v>
       </c>
       <c r="J19" s="84" t="n">
-        <v>32.05</v>
+        <v>31.65</v>
       </c>
       <c r="K19" s="88" t="n">
         <v>64.09999999999999</v>
@@ -30442,12 +30442,12 @@
       </c>
       <c r="B23" s="83" t="inlineStr">
         <is>
-          <t>Union Balanced Advantage Fund - Regular Plan - Growth Option</t>
+          <t>Axis Balanced Advantage Fund - Regular Plan - Growth</t>
         </is>
       </c>
       <c r="C23" s="83" t="inlineStr">
         <is>
-          <t>Union Mutual Fund</t>
+          <t>Axis Mutual Fund</t>
         </is>
       </c>
       <c r="D23" s="83" t="inlineStr">
@@ -30456,22 +30456,22 @@
         </is>
       </c>
       <c r="E23" s="84" t="n">
-        <v>1.8</v>
+        <v>1.67</v>
       </c>
       <c r="F23" s="84" t="n">
-        <v>5.83</v>
+        <v>5.37</v>
       </c>
       <c r="G23" s="86" t="n">
-        <v>-1.07</v>
+        <v>-0.88</v>
       </c>
       <c r="H23" s="84" t="n">
-        <v>0.1</v>
+        <v>1.09</v>
       </c>
       <c r="I23" s="84" t="n">
-        <v>2.4987804805501</v>
+        <v>4.713895925994471</v>
       </c>
       <c r="J23" s="84" t="n">
-        <v>26.65</v>
+        <v>40.96</v>
       </c>
       <c r="K23" s="88" t="n">
         <v>57.8</v>
@@ -30509,12 +30509,12 @@
       </c>
       <c r="B24" s="79" t="inlineStr">
         <is>
-          <t>Axis Balanced Advantage Fund - Regular Plan - Growth</t>
+          <t>Union Balanced Advantage Fund - Regular Plan - Growth Option</t>
         </is>
       </c>
       <c r="C24" s="79" t="inlineStr">
         <is>
-          <t>Axis Mutual Fund</t>
+          <t>Union Mutual Fund</t>
         </is>
       </c>
       <c r="D24" s="79" t="inlineStr">
@@ -30523,22 +30523,22 @@
         </is>
       </c>
       <c r="E24" s="80" t="n">
-        <v>1.67</v>
+        <v>1.8</v>
       </c>
       <c r="F24" s="80" t="n">
-        <v>5.37</v>
+        <v>5.83</v>
       </c>
       <c r="G24" s="87" t="n">
-        <v>-0.88</v>
+        <v>-1.07</v>
       </c>
       <c r="H24" s="80" t="n">
-        <v>1.09</v>
+        <v>0.1</v>
       </c>
       <c r="I24" s="80" t="n">
-        <v>4.713895925994471</v>
+        <v>2.4987804805501</v>
       </c>
       <c r="J24" s="80" t="n">
-        <v>40.96</v>
+        <v>26.65</v>
       </c>
       <c r="K24" s="88" t="n">
         <v>57.8</v>
@@ -31514,12 +31514,12 @@
       </c>
       <c r="B39" s="83" t="inlineStr">
         <is>
-          <t>ITI Balanced Advantage Fund - Regular Plan - Growth Option</t>
+          <t>PGIM India Balanced Advantage Fund - Regular Plan - Growth Option</t>
         </is>
       </c>
       <c r="C39" s="83" t="inlineStr">
         <is>
-          <t>ITI Mutual Fund</t>
+          <t>PGIM India Mutual Fund</t>
         </is>
       </c>
       <c r="D39" s="83" t="inlineStr">
@@ -31528,22 +31528,22 @@
         </is>
       </c>
       <c r="E39" s="84" t="n">
-        <v>1.11</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="F39" s="84" t="n">
-        <v>4.28</v>
+        <v>5.64</v>
       </c>
       <c r="G39" s="86" t="n">
-        <v>-3.66</v>
+        <v>-3.29</v>
       </c>
       <c r="H39" s="86" t="n">
-        <v>-2.89</v>
+        <v>-3.97</v>
       </c>
       <c r="I39" s="84" t="n">
-        <v>1.602165331256589</v>
+        <v>1.533245786786508</v>
       </c>
       <c r="J39" s="84" t="n">
-        <v>27.39</v>
+        <v>21.18</v>
       </c>
       <c r="K39" s="89" t="n">
         <v>25.1</v>
@@ -31581,12 +31581,12 @@
       </c>
       <c r="B40" s="79" t="inlineStr">
         <is>
-          <t>PGIM India Balanced Advantage Fund - Regular Plan - Growth Option</t>
+          <t>ITI Balanced Advantage Fund - Regular Plan - Growth Option</t>
         </is>
       </c>
       <c r="C40" s="79" t="inlineStr">
         <is>
-          <t>PGIM India Mutual Fund</t>
+          <t>ITI Mutual Fund</t>
         </is>
       </c>
       <c r="D40" s="79" t="inlineStr">
@@ -31595,22 +31595,22 @@
         </is>
       </c>
       <c r="E40" s="80" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.11</v>
       </c>
       <c r="F40" s="80" t="n">
-        <v>5.64</v>
+        <v>4.28</v>
       </c>
       <c r="G40" s="87" t="n">
-        <v>-3.29</v>
+        <v>-3.66</v>
       </c>
       <c r="H40" s="87" t="n">
-        <v>-3.97</v>
+        <v>-2.89</v>
       </c>
       <c r="I40" s="80" t="n">
-        <v>1.533245786786508</v>
+        <v>1.602165331256589</v>
       </c>
       <c r="J40" s="80" t="n">
-        <v>21.18</v>
+        <v>27.39</v>
       </c>
       <c r="K40" s="89" t="n">
         <v>25.1</v>
@@ -33647,7 +33647,7 @@
       </c>
       <c r="B26" s="79" t="inlineStr">
         <is>
-          <t>Nippon India Equity Savings Fund- Growth Plan- Growth Option</t>
+          <t>Nippon India Equity Savings Fund- Growth Plan- Bonus Option</t>
         </is>
       </c>
       <c r="C26" s="79" t="inlineStr">
@@ -33714,7 +33714,7 @@
       </c>
       <c r="B27" s="83" t="inlineStr">
         <is>
-          <t>Nippon India Equity Savings Fund- Growth Plan- Bonus Option</t>
+          <t>Nippon India Equity Savings Fund- Growth Plan- Growth Option</t>
         </is>
       </c>
       <c r="C27" s="83" t="inlineStr">
@@ -34842,12 +34842,12 @@
       </c>
       <c r="B13" s="26" t="inlineStr">
         <is>
-          <t>HSBC Multi Asset Allocation Fund - Regular - Growth</t>
+          <t>Union Multi Asset Allocation Fund- Regular Plan - Growth Option</t>
         </is>
       </c>
       <c r="C13" s="26" t="inlineStr">
         <is>
-          <t>HSBC Mutual Fund</t>
+          <t>Union Mutual Fund</t>
         </is>
       </c>
       <c r="D13" s="26" t="inlineStr">
@@ -34855,20 +34855,20 @@
           <t>Multi Asset Allocation</t>
         </is>
       </c>
-      <c r="E13" s="97" t="n">
-        <v>-1.36</v>
+      <c r="E13" s="27" t="n">
+        <v>0.33</v>
       </c>
       <c r="F13" s="27" t="n">
-        <v>8.630000000000001</v>
+        <v>6.08</v>
       </c>
       <c r="G13" s="27" t="n">
-        <v>3.82</v>
+        <v>1.6</v>
       </c>
       <c r="H13" s="27" t="n">
-        <v>15.3</v>
+        <v>12.32</v>
       </c>
       <c r="I13" s="27" t="n">
-        <v>9.781601372907666</v>
+        <v>0</v>
       </c>
       <c r="J13" s="27" t="n">
         <v>0</v>
@@ -34909,12 +34909,12 @@
       </c>
       <c r="B14" s="26" t="inlineStr">
         <is>
-          <t>Union Multi Asset Allocation Fund- Regular Plan - Growth Option</t>
+          <t>HSBC Multi Asset Allocation Fund - Regular - Growth</t>
         </is>
       </c>
       <c r="C14" s="26" t="inlineStr">
         <is>
-          <t>Union Mutual Fund</t>
+          <t>HSBC Mutual Fund</t>
         </is>
       </c>
       <c r="D14" s="26" t="inlineStr">
@@ -34922,20 +34922,20 @@
           <t>Multi Asset Allocation</t>
         </is>
       </c>
-      <c r="E14" s="27" t="n">
-        <v>0.33</v>
+      <c r="E14" s="97" t="n">
+        <v>-1.36</v>
       </c>
       <c r="F14" s="27" t="n">
-        <v>6.08</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="G14" s="27" t="n">
-        <v>1.6</v>
+        <v>3.82</v>
       </c>
       <c r="H14" s="27" t="n">
-        <v>12.32</v>
+        <v>15.3</v>
       </c>
       <c r="I14" s="27" t="n">
-        <v>0</v>
+        <v>9.781601372907666</v>
       </c>
       <c r="J14" s="27" t="n">
         <v>0</v>

</xml_diff>